<commit_message>
feat: Implementação do Menor Preço e remoção de redundância frontend/backend
</commit_message>
<xml_diff>
--- a/tenisideal-catalogo atualizada.xlsx
+++ b/tenisideal-catalogo atualizada.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cristianamoreira/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cristianamoreira/Desktop/tenisideal/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C33ECDE-24BC-CE43-9C25-431C4D29D303}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D6C7EEC-ACFB-3C4C-9E6A-DCDD9E970932}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="25600" windowHeight="14360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="25600" windowHeight="14300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Catálogo" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1422" uniqueCount="661">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1459" uniqueCount="677">
   <si>
     <t>PRODUTO</t>
   </si>
@@ -961,19 +961,10 @@
     <t>Pegasus 41</t>
   </si>
   <si>
-    <t>https://images-na.ssl-images-amazon.com/images/I/71r5ZHElneL.jpg</t>
-  </si>
-  <si>
     <t>Clássico|Versátil</t>
   </si>
   <si>
-    <t>R$1.346</t>
-  </si>
-  <si>
     <t>O tênis de corrida mais vendido do mundo. Versátil, durável e confortável para qualquer treino.</t>
-  </si>
-  <si>
-    <t>https://amzn.to/4bnDb44</t>
   </si>
   <si>
     <t>Reactx Infinity Run 4</t>
@@ -2015,15 +2006,252 @@
   <si>
     <t>10 x R$ 59,99 sem juros</t>
   </si>
+  <si>
+    <r>
+      <t>R$ 664,99</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> no Pix</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>7x</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF111111"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t> de R$</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color rgb="FF111111"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t> 100,00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF111111"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t> sem juros</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>R$ 683,99</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="1"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t> n</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>no Pix</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>7x</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF111111"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t> de </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color rgb="FF111111"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t>R$ 102,86</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF111111"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t> sem juros</t>
+    </r>
+  </si>
+  <si>
+    <t>https://m.media-amazon.com/images/I/71I5TWi+77L._AC_SY500_.jpg</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4lMlD5y</t>
+  </si>
+  <si>
+    <t>https://tidd.ly/47bxsfp</t>
+  </si>
+  <si>
+    <t>https://m.media-amazon.com/images/I/51uEAp-HMPL._AC_SY500_.jpg</t>
+  </si>
+  <si>
+    <r>
+      <t>R$</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="28"/>
+        <color rgb="FF0F1111"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>728,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF0F1111"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>08</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF0F1111"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+  </si>
+  <si>
+    <t>https://amzn.to/40D0qkP</t>
+  </si>
+  <si>
+    <t>https://tidd.ly/4lAM120</t>
+  </si>
+  <si>
+    <t>Vomero Plus</t>
+  </si>
+  <si>
+    <t>https://imgnike-a.akamaihd.net/1920x1920/05924154A2.jpg</t>
+  </si>
+  <si>
+    <r>
+      <t>10x</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF111111"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t> de </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color rgb="FF111111"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t>R$ 130,00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF111111"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t> sem juros</t>
+    </r>
+  </si>
+  <si>
+    <t>https://tidd.ly/3PaPl86</t>
+  </si>
+  <si>
+    <t>https://imgnike-a.akamaihd.net/360x360/059366NEA2.jpg</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4dt98th</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4cXLGEl</t>
+  </si>
+  <si>
+    <r>
+      <t>R$</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="28"/>
+        <color rgb="FF0F1111"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>1.813,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF0F1111"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>66</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF0F1111"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="6" formatCode="&quot;R$&quot;\ #,##0;[Red]\-&quot;R$&quot;\ #,##0"/>
     <numFmt numFmtId="8" formatCode="&quot;R$&quot;\ #,##0.00;[Red]\-&quot;R$&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2087,6 +2315,49 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Whitney-Medium"/>
+    </font>
+    <font>
+      <sz val="1"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF111111"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF111111"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="28"/>
+      <color rgb="FF0F1111"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color rgb="FF0F1111"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF0F1111"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="9">
@@ -2158,7 +2429,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2185,16 +2456,6 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -2214,6 +2475,25 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="6" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
@@ -2517,7 +2797,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R95"/>
+  <dimension ref="A1:R98"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -2538,31 +2818,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="22" customHeight="1">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="13" t="s">
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="12" t="s">
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="K1" s="11"/>
-      <c r="L1" s="11"/>
-      <c r="M1" s="11"/>
-      <c r="N1" s="11"/>
-      <c r="O1" s="11"/>
-      <c r="P1" s="10" t="s">
+      <c r="K1" s="18"/>
+      <c r="L1" s="18"/>
+      <c r="M1" s="18"/>
+      <c r="N1" s="18"/>
+      <c r="O1" s="18"/>
+      <c r="P1" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="Q1" s="11"/>
+      <c r="Q1" s="18"/>
       <c r="R1" s="1"/>
     </row>
     <row r="2" spans="1:18" ht="18" customHeight="1">
@@ -2640,14 +2920,14 @@
       <c r="F3" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="G3" s="18" t="s">
-        <v>633</v>
-      </c>
-      <c r="H3" s="15">
+      <c r="G3" s="14" t="s">
+        <v>630</v>
+      </c>
+      <c r="H3" s="11">
         <v>1999.99</v>
       </c>
-      <c r="I3" s="15" t="s">
-        <v>632</v>
+      <c r="I3" s="11" t="s">
+        <v>629</v>
       </c>
       <c r="J3" s="5" t="s">
         <v>28</v>
@@ -2667,10 +2947,10 @@
       <c r="O3" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="P3" s="16" t="s">
+      <c r="P3" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="Q3" s="14" t="s">
+      <c r="Q3" s="10" t="s">
         <v>35</v>
       </c>
       <c r="R3" s="5"/>
@@ -2694,14 +2974,14 @@
       <c r="F4" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="G4" s="19">
+      <c r="G4" s="15">
         <v>1313.78</v>
       </c>
-      <c r="H4" s="15">
+      <c r="H4" s="11">
         <v>1399.99</v>
       </c>
-      <c r="I4" s="15" t="s">
-        <v>635</v>
+      <c r="I4" s="11" t="s">
+        <v>632</v>
       </c>
       <c r="J4" s="5" t="s">
         <v>28</v>
@@ -2721,10 +3001,10 @@
       <c r="O4" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="P4" s="16" t="s">
+      <c r="P4" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="Q4" s="14" t="s">
+      <c r="Q4" s="10" t="s">
         <v>43</v>
       </c>
       <c r="R4" s="5"/>
@@ -2748,14 +3028,14 @@
       <c r="F5" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="G5" s="17">
+      <c r="G5" s="13">
         <v>399.88</v>
       </c>
-      <c r="H5" s="15">
+      <c r="H5" s="11">
         <v>399.99</v>
       </c>
-      <c r="I5" s="15" t="s">
-        <v>634</v>
+      <c r="I5" s="11" t="s">
+        <v>631</v>
       </c>
       <c r="J5" s="5" t="s">
         <v>48</v>
@@ -2775,10 +3055,10 @@
       <c r="O5" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="P5" s="16" t="s">
+      <c r="P5" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="Q5" s="14" t="s">
+      <c r="Q5" s="10" t="s">
         <v>54</v>
       </c>
       <c r="R5" s="5"/>
@@ -2802,14 +3082,14 @@
       <c r="F6" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="G6" s="17">
+      <c r="G6" s="13">
         <v>945.11</v>
       </c>
-      <c r="H6" s="15">
+      <c r="H6" s="11">
         <v>1099.99</v>
       </c>
-      <c r="I6" s="15" t="s">
-        <v>636</v>
+      <c r="I6" s="11" t="s">
+        <v>633</v>
       </c>
       <c r="J6" s="5" t="s">
         <v>28</v>
@@ -2829,10 +3109,10 @@
       <c r="O6" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="P6" s="16" t="s">
+      <c r="P6" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="Q6" s="14" t="s">
+      <c r="Q6" s="10" t="s">
         <v>61</v>
       </c>
       <c r="R6" s="5"/>
@@ -2854,14 +3134,14 @@
         <v>26</v>
       </c>
       <c r="F7" s="5"/>
-      <c r="G7" s="19" t="s">
+      <c r="G7" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="H7" s="15">
+      <c r="H7" s="11">
         <v>1199.99</v>
       </c>
-      <c r="I7" s="15" t="s">
-        <v>637</v>
+      <c r="I7" s="11" t="s">
+        <v>634</v>
       </c>
       <c r="J7" s="5" t="s">
         <v>28</v>
@@ -2871,10 +3151,10 @@
       <c r="M7" s="5"/>
       <c r="N7" s="5"/>
       <c r="O7" s="5"/>
-      <c r="P7" s="16" t="s">
+      <c r="P7" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="Q7" s="14" t="s">
+      <c r="Q7" s="10" t="s">
         <v>66</v>
       </c>
       <c r="R7" s="5"/>
@@ -2901,11 +3181,11 @@
       <c r="G8" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="H8" s="15">
+      <c r="H8" s="11">
         <v>1099.99</v>
       </c>
-      <c r="I8" s="15" t="s">
-        <v>639</v>
+      <c r="I8" s="11" t="s">
+        <v>636</v>
       </c>
       <c r="J8" s="5" t="s">
         <v>28</v>
@@ -2925,10 +3205,10 @@
       <c r="O8" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="P8" s="16" t="s">
+      <c r="P8" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="Q8" s="14" t="s">
+      <c r="Q8" s="10" t="s">
         <v>73</v>
       </c>
       <c r="R8" s="5"/>
@@ -2955,11 +3235,11 @@
       <c r="G9" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="H9" s="15">
+      <c r="H9" s="11">
         <v>599.99</v>
       </c>
-      <c r="I9" s="15" t="s">
-        <v>638</v>
+      <c r="I9" s="11" t="s">
+        <v>635</v>
       </c>
       <c r="J9" s="5" t="s">
         <v>48</v>
@@ -2979,10 +3259,10 @@
       <c r="O9" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="P9" s="16" t="s">
+      <c r="P9" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="Q9" s="14" t="s">
+      <c r="Q9" s="10" t="s">
         <v>82</v>
       </c>
       <c r="R9" s="5"/>
@@ -3009,11 +3289,11 @@
       <c r="G10" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="H10" s="15">
+      <c r="H10" s="11">
         <v>1199.99</v>
       </c>
-      <c r="I10" s="15" t="s">
-        <v>641</v>
+      <c r="I10" s="11" t="s">
+        <v>638</v>
       </c>
       <c r="J10" s="5" t="s">
         <v>28</v>
@@ -3033,11 +3313,11 @@
       <c r="O10" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="P10" s="16" t="s">
+      <c r="P10" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="Q10" s="14" t="s">
-        <v>640</v>
+      <c r="Q10" s="10" t="s">
+        <v>637</v>
       </c>
       <c r="R10" s="5"/>
     </row>
@@ -4247,11 +4527,11 @@
       <c r="G35" s="6" t="s">
         <v>251</v>
       </c>
-      <c r="H35" s="15">
+      <c r="H35" s="11">
         <v>649.99</v>
       </c>
-      <c r="I35" s="15" t="s">
-        <v>642</v>
+      <c r="I35" s="11" t="s">
+        <v>639</v>
       </c>
       <c r="J35" s="5" t="s">
         <v>98</v>
@@ -4271,7 +4551,7 @@
       <c r="O35" s="5" t="s">
         <v>252</v>
       </c>
-      <c r="P35" s="16" t="s">
+      <c r="P35" s="12" t="s">
         <v>253</v>
       </c>
       <c r="Q35" s="8" t="s">
@@ -4301,11 +4581,11 @@
       <c r="G36" s="6" t="s">
         <v>258</v>
       </c>
-      <c r="H36" s="15">
+      <c r="H36" s="11">
         <v>549.99</v>
       </c>
-      <c r="I36" s="15" t="s">
-        <v>643</v>
+      <c r="I36" s="11" t="s">
+        <v>640</v>
       </c>
       <c r="J36" s="5" t="s">
         <v>48</v>
@@ -4355,11 +4635,11 @@
       <c r="G37" s="6" t="s">
         <v>266</v>
       </c>
-      <c r="H37" s="15">
+      <c r="H37" s="11">
         <v>1199.99</v>
       </c>
-      <c r="I37" s="15" t="s">
-        <v>644</v>
+      <c r="I37" s="11" t="s">
+        <v>641</v>
       </c>
       <c r="J37" s="5" t="s">
         <v>28</v>
@@ -4409,11 +4689,11 @@
       <c r="G38" s="6" t="s">
         <v>273</v>
       </c>
-      <c r="H38" s="15">
+      <c r="H38" s="11">
         <v>329.99</v>
       </c>
-      <c r="I38" s="15" t="s">
-        <v>645</v>
+      <c r="I38" s="11" t="s">
+        <v>642</v>
       </c>
       <c r="J38" s="5" t="s">
         <v>48</v>
@@ -4754,21 +5034,25 @@
         <v>312</v>
       </c>
       <c r="D45" s="5" t="s">
+        <v>662</v>
+      </c>
+      <c r="E45" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F45" s="5" t="s">
         <v>313</v>
       </c>
-      <c r="E45" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="F45" s="5" t="s">
-        <v>314</v>
-      </c>
-      <c r="G45" s="6" t="s">
-        <v>315</v>
-      </c>
-      <c r="H45" s="9"/>
-      <c r="I45" s="9"/>
+      <c r="G45" s="21">
+        <v>844.61</v>
+      </c>
+      <c r="H45" s="11" t="s">
+        <v>658</v>
+      </c>
+      <c r="I45" s="11" t="s">
+        <v>659</v>
+      </c>
       <c r="J45" s="5" t="s">
-        <v>28</v>
+        <v>98</v>
       </c>
       <c r="K45" s="5" t="s">
         <v>88</v>
@@ -4783,13 +5067,13 @@
         <v>51</v>
       </c>
       <c r="O45" s="5" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="P45" s="6" t="s">
-        <v>317</v>
-      </c>
-      <c r="Q45" s="5" t="s">
-        <v>102</v>
+        <v>663</v>
+      </c>
+      <c r="Q45" s="8" t="s">
+        <v>664</v>
       </c>
       <c r="R45" s="5" t="s">
         <v>103</v>
@@ -4797,33 +5081,37 @@
     </row>
     <row r="46" spans="1:18" ht="18" customHeight="1">
       <c r="A46" s="5" t="s">
-        <v>22</v>
+        <v>67</v>
       </c>
       <c r="B46" s="5" t="s">
         <v>311</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>319</v>
+        <v>665</v>
       </c>
       <c r="E46" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F46" s="5" t="s">
-        <v>320</v>
-      </c>
-      <c r="G46" s="6" t="s">
-        <v>321</v>
-      </c>
-      <c r="H46" s="9"/>
-      <c r="I46" s="9"/>
+        <v>313</v>
+      </c>
+      <c r="G46" s="21" t="s">
+        <v>666</v>
+      </c>
+      <c r="H46" s="11" t="s">
+        <v>660</v>
+      </c>
+      <c r="I46" s="11" t="s">
+        <v>661</v>
+      </c>
       <c r="J46" s="5" t="s">
-        <v>28</v>
+        <v>98</v>
       </c>
       <c r="K46" s="5" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="L46" s="5" t="s">
         <v>50</v>
@@ -4832,40 +5120,40 @@
         <v>31</v>
       </c>
       <c r="N46" s="5" t="s">
-        <v>109</v>
+        <v>51</v>
       </c>
       <c r="O46" s="5" t="s">
-        <v>322</v>
+        <v>314</v>
       </c>
       <c r="P46" s="6" t="s">
-        <v>323</v>
-      </c>
-      <c r="Q46" s="5" t="s">
-        <v>102</v>
+        <v>667</v>
+      </c>
+      <c r="Q46" s="8" t="s">
+        <v>668</v>
       </c>
       <c r="R46" s="5"/>
     </row>
     <row r="47" spans="1:18" ht="18" customHeight="1">
       <c r="A47" s="5" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="B47" s="5" t="s">
         <v>311</v>
       </c>
       <c r="C47" s="5" t="s">
+        <v>315</v>
+      </c>
+      <c r="D47" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="E47" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F47" s="5" t="s">
+        <v>317</v>
+      </c>
+      <c r="G47" s="6" t="s">
         <v>318</v>
-      </c>
-      <c r="D47" s="5" t="s">
-        <v>324</v>
-      </c>
-      <c r="E47" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="F47" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="G47" s="6" t="s">
-        <v>326</v>
       </c>
       <c r="H47" s="9"/>
       <c r="I47" s="9"/>
@@ -4885,10 +5173,10 @@
         <v>109</v>
       </c>
       <c r="O47" s="5" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="P47" s="6" t="s">
-        <v>327</v>
+        <v>320</v>
       </c>
       <c r="Q47" s="5" t="s">
         <v>102</v>
@@ -4897,25 +5185,25 @@
     </row>
     <row r="48" spans="1:18" ht="18" customHeight="1">
       <c r="A48" s="5" t="s">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="B48" s="5" t="s">
         <v>311</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>328</v>
+        <v>315</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>329</v>
+        <v>321</v>
       </c>
       <c r="E48" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F48" s="5" t="s">
-        <v>330</v>
+        <v>322</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>331</v>
+        <v>323</v>
       </c>
       <c r="H48" s="9"/>
       <c r="I48" s="9"/>
@@ -4923,22 +5211,22 @@
         <v>28</v>
       </c>
       <c r="K48" s="5" t="s">
-        <v>29</v>
+        <v>78</v>
       </c>
       <c r="L48" s="5" t="s">
-        <v>332</v>
+        <v>50</v>
       </c>
       <c r="M48" s="5" t="s">
         <v>31</v>
       </c>
       <c r="N48" s="5" t="s">
-        <v>32</v>
+        <v>109</v>
       </c>
       <c r="O48" s="5" t="s">
-        <v>333</v>
+        <v>319</v>
       </c>
       <c r="P48" s="6" t="s">
-        <v>334</v>
+        <v>324</v>
       </c>
       <c r="Q48" s="5" t="s">
         <v>102</v>
@@ -4953,19 +5241,19 @@
         <v>311</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>335</v>
+        <v>325</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>336</v>
+        <v>326</v>
       </c>
       <c r="E49" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F49" s="5" t="s">
-        <v>337</v>
+        <v>327</v>
       </c>
       <c r="G49" s="6" t="s">
-        <v>338</v>
+        <v>328</v>
       </c>
       <c r="H49" s="9"/>
       <c r="I49" s="9"/>
@@ -4976,19 +5264,19 @@
         <v>29</v>
       </c>
       <c r="L49" s="5" t="s">
-        <v>30</v>
+        <v>329</v>
       </c>
       <c r="M49" s="5" t="s">
-        <v>339</v>
+        <v>31</v>
       </c>
       <c r="N49" s="5" t="s">
         <v>32</v>
       </c>
       <c r="O49" s="5" t="s">
-        <v>340</v>
+        <v>330</v>
       </c>
       <c r="P49" s="6" t="s">
-        <v>341</v>
+        <v>331</v>
       </c>
       <c r="Q49" s="5" t="s">
         <v>102</v>
@@ -5000,48 +5288,40 @@
         <v>22</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>342</v>
+        <v>311</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>343</v>
+        <v>669</v>
       </c>
       <c r="D50" s="5" t="s">
-        <v>344</v>
+        <v>670</v>
       </c>
       <c r="E50" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="F50" s="5" t="s">
-        <v>345</v>
-      </c>
-      <c r="G50" s="6" t="s">
-        <v>346</v>
-      </c>
-      <c r="H50" s="9"/>
-      <c r="I50" s="9"/>
+      <c r="F50" s="5"/>
+      <c r="G50" s="22">
+        <v>1860.73</v>
+      </c>
+      <c r="H50" s="23">
+        <v>1234.99</v>
+      </c>
+      <c r="I50" s="11" t="s">
+        <v>671</v>
+      </c>
       <c r="J50" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="K50" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="L50" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="M50" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="N50" s="5" t="s">
-        <v>283</v>
-      </c>
-      <c r="O50" s="5" t="s">
-        <v>347</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="K50" s="5"/>
+      <c r="L50" s="5"/>
+      <c r="M50" s="5"/>
+      <c r="N50" s="5"/>
+      <c r="O50" s="5"/>
       <c r="P50" s="6" t="s">
-        <v>348</v>
-      </c>
-      <c r="Q50" s="5" t="s">
-        <v>102</v>
+        <v>674</v>
+      </c>
+      <c r="Q50" s="10" t="s">
+        <v>672</v>
       </c>
       <c r="R50" s="5"/>
     </row>
@@ -5050,48 +5330,40 @@
         <v>67</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>342</v>
+        <v>311</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>349</v>
+        <v>669</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>350</v>
+        <v>673</v>
       </c>
       <c r="E51" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="F51" s="5" t="s">
-        <v>345</v>
-      </c>
-      <c r="G51" s="6" t="s">
-        <v>351</v>
-      </c>
-      <c r="H51" s="9"/>
-      <c r="I51" s="9"/>
+      <c r="F51" s="5"/>
+      <c r="G51" s="22" t="s">
+        <v>676</v>
+      </c>
+      <c r="H51" s="23">
+        <v>1234.99</v>
+      </c>
+      <c r="I51" s="11" t="s">
+        <v>671</v>
+      </c>
       <c r="J51" s="5" t="s">
-        <v>204</v>
-      </c>
-      <c r="K51" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="L51" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="M51" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="N51" s="5" t="s">
-        <v>283</v>
-      </c>
-      <c r="O51" s="5" t="s">
-        <v>352</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="K51" s="5"/>
+      <c r="L51" s="5"/>
+      <c r="M51" s="5"/>
+      <c r="N51" s="5"/>
+      <c r="O51" s="5"/>
       <c r="P51" s="6" t="s">
-        <v>353</v>
-      </c>
-      <c r="Q51" s="5" t="s">
-        <v>102</v>
+        <v>675</v>
+      </c>
+      <c r="Q51" s="10" t="s">
+        <v>668</v>
       </c>
       <c r="R51" s="5"/>
     </row>
@@ -5100,47 +5372,49 @@
         <v>22</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>342</v>
+        <v>311</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>354</v>
+        <v>332</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>355</v>
+        <v>333</v>
       </c>
       <c r="E52" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F52" s="5" t="s">
-        <v>356</v>
+        <v>334</v>
       </c>
       <c r="G52" s="6" t="s">
-        <v>357</v>
+        <v>335</v>
       </c>
       <c r="H52" s="9"/>
       <c r="I52" s="9"/>
       <c r="J52" s="5" t="s">
-        <v>204</v>
+        <v>28</v>
       </c>
       <c r="K52" s="5" t="s">
-        <v>78</v>
+        <v>29</v>
       </c>
       <c r="L52" s="5" t="s">
         <v>30</v>
       </c>
       <c r="M52" s="5" t="s">
-        <v>89</v>
+        <v>336</v>
       </c>
       <c r="N52" s="5" t="s">
-        <v>99</v>
+        <v>32</v>
       </c>
       <c r="O52" s="5" t="s">
-        <v>358</v>
+        <v>337</v>
       </c>
       <c r="P52" s="6" t="s">
-        <v>359</v>
-      </c>
-      <c r="Q52" s="5"/>
+        <v>338</v>
+      </c>
+      <c r="Q52" s="5" t="s">
+        <v>102</v>
+      </c>
       <c r="R52" s="5"/>
     </row>
     <row r="53" spans="1:18" ht="18" customHeight="1">
@@ -5148,47 +5422,49 @@
         <v>22</v>
       </c>
       <c r="B53" s="5" t="s">
+        <v>339</v>
+      </c>
+      <c r="C53" s="5" t="s">
+        <v>340</v>
+      </c>
+      <c r="D53" s="5" t="s">
+        <v>341</v>
+      </c>
+      <c r="E53" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F53" s="5" t="s">
         <v>342</v>
       </c>
-      <c r="C53" s="5" t="s">
-        <v>360</v>
-      </c>
-      <c r="D53" s="5" t="s">
-        <v>361</v>
-      </c>
-      <c r="E53" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="F53" s="5" t="s">
-        <v>362</v>
-      </c>
       <c r="G53" s="6" t="s">
-        <v>363</v>
+        <v>343</v>
       </c>
       <c r="H53" s="9"/>
       <c r="I53" s="9"/>
       <c r="J53" s="5" t="s">
-        <v>204</v>
+        <v>48</v>
       </c>
       <c r="K53" s="5" t="s">
         <v>49</v>
       </c>
       <c r="L53" s="5" t="s">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="M53" s="5" t="s">
-        <v>89</v>
+        <v>31</v>
       </c>
       <c r="N53" s="5" t="s">
-        <v>79</v>
+        <v>283</v>
       </c>
       <c r="O53" s="5" t="s">
-        <v>364</v>
+        <v>344</v>
       </c>
       <c r="P53" s="6" t="s">
-        <v>365</v>
-      </c>
-      <c r="Q53" s="5"/>
+        <v>345</v>
+      </c>
+      <c r="Q53" s="5" t="s">
+        <v>102</v>
+      </c>
       <c r="R53" s="5"/>
     </row>
     <row r="54" spans="1:18" ht="18" customHeight="1">
@@ -5196,22 +5472,22 @@
         <v>67</v>
       </c>
       <c r="B54" s="5" t="s">
+        <v>339</v>
+      </c>
+      <c r="C54" s="5" t="s">
+        <v>346</v>
+      </c>
+      <c r="D54" s="5" t="s">
+        <v>347</v>
+      </c>
+      <c r="E54" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F54" s="5" t="s">
         <v>342</v>
       </c>
-      <c r="C54" s="5" t="s">
-        <v>366</v>
-      </c>
-      <c r="D54" s="5" t="s">
-        <v>367</v>
-      </c>
-      <c r="E54" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="F54" s="5" t="s">
-        <v>368</v>
-      </c>
       <c r="G54" s="6" t="s">
-        <v>357</v>
+        <v>348</v>
       </c>
       <c r="H54" s="9"/>
       <c r="I54" s="9"/>
@@ -5219,47 +5495,49 @@
         <v>204</v>
       </c>
       <c r="K54" s="5" t="s">
-        <v>78</v>
+        <v>49</v>
       </c>
       <c r="L54" s="5" t="s">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="M54" s="5" t="s">
-        <v>89</v>
+        <v>31</v>
       </c>
       <c r="N54" s="5" t="s">
-        <v>369</v>
+        <v>283</v>
       </c>
       <c r="O54" s="5" t="s">
-        <v>370</v>
+        <v>349</v>
       </c>
       <c r="P54" s="6" t="s">
-        <v>371</v>
-      </c>
-      <c r="Q54" s="5"/>
+        <v>350</v>
+      </c>
+      <c r="Q54" s="5" t="s">
+        <v>102</v>
+      </c>
       <c r="R54" s="5"/>
     </row>
     <row r="55" spans="1:18" ht="18" customHeight="1">
       <c r="A55" s="5" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>372</v>
+        <v>351</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>373</v>
+        <v>352</v>
       </c>
       <c r="E55" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F55" s="5" t="s">
-        <v>374</v>
+        <v>353</v>
       </c>
       <c r="G55" s="6" t="s">
-        <v>375</v>
+        <v>354</v>
       </c>
       <c r="H55" s="9"/>
       <c r="I55" s="9"/>
@@ -5276,13 +5554,13 @@
         <v>89</v>
       </c>
       <c r="N55" s="5" t="s">
-        <v>376</v>
+        <v>99</v>
       </c>
       <c r="O55" s="5" t="s">
-        <v>377</v>
+        <v>355</v>
       </c>
       <c r="P55" s="6" t="s">
-        <v>378</v>
+        <v>356</v>
       </c>
       <c r="Q55" s="5"/>
       <c r="R55" s="5"/>
@@ -5292,72 +5570,70 @@
         <v>22</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>379</v>
+        <v>339</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>380</v>
+        <v>357</v>
       </c>
       <c r="D56" s="5" t="s">
-        <v>381</v>
+        <v>358</v>
       </c>
       <c r="E56" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F56" s="5" t="s">
-        <v>382</v>
+        <v>359</v>
       </c>
       <c r="G56" s="6" t="s">
-        <v>383</v>
+        <v>360</v>
       </c>
       <c r="H56" s="9"/>
       <c r="I56" s="9"/>
       <c r="J56" s="5" t="s">
-        <v>98</v>
+        <v>204</v>
       </c>
       <c r="K56" s="5" t="s">
-        <v>78</v>
+        <v>49</v>
       </c>
       <c r="L56" s="5" t="s">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="M56" s="5" t="s">
-        <v>31</v>
+        <v>89</v>
       </c>
       <c r="N56" s="5" t="s">
         <v>79</v>
       </c>
       <c r="O56" s="5" t="s">
-        <v>384</v>
+        <v>361</v>
       </c>
       <c r="P56" s="6" t="s">
-        <v>385</v>
-      </c>
-      <c r="Q56" s="5" t="s">
-        <v>102</v>
-      </c>
+        <v>362</v>
+      </c>
+      <c r="Q56" s="5"/>
       <c r="R56" s="5"/>
     </row>
     <row r="57" spans="1:18" ht="18" customHeight="1">
       <c r="A57" s="5" t="s">
-        <v>44</v>
+        <v>67</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>379</v>
+        <v>339</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>386</v>
+        <v>363</v>
       </c>
       <c r="D57" s="5" t="s">
-        <v>387</v>
+        <v>364</v>
       </c>
       <c r="E57" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F57" s="5" t="s">
-        <v>86</v>
+        <v>365</v>
       </c>
       <c r="G57" s="6" t="s">
-        <v>388</v>
+        <v>354</v>
       </c>
       <c r="H57" s="9"/>
       <c r="I57" s="9"/>
@@ -5374,65 +5650,63 @@
         <v>89</v>
       </c>
       <c r="N57" s="5" t="s">
-        <v>90</v>
+        <v>366</v>
       </c>
       <c r="O57" s="5" t="s">
-        <v>389</v>
+        <v>367</v>
       </c>
       <c r="P57" s="6" t="s">
-        <v>390</v>
+        <v>368</v>
       </c>
       <c r="Q57" s="5"/>
       <c r="R57" s="5"/>
     </row>
     <row r="58" spans="1:18" ht="18" customHeight="1">
       <c r="A58" s="5" t="s">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>391</v>
+        <v>339</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>392</v>
+        <v>369</v>
       </c>
       <c r="D58" s="5" t="s">
-        <v>393</v>
+        <v>370</v>
       </c>
       <c r="E58" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F58" s="5" t="s">
-        <v>394</v>
+        <v>371</v>
       </c>
       <c r="G58" s="6" t="s">
-        <v>395</v>
+        <v>372</v>
       </c>
       <c r="H58" s="9"/>
       <c r="I58" s="9"/>
       <c r="J58" s="5" t="s">
-        <v>28</v>
+        <v>204</v>
       </c>
       <c r="K58" s="5" t="s">
-        <v>39</v>
+        <v>78</v>
       </c>
       <c r="L58" s="5" t="s">
-        <v>332</v>
+        <v>30</v>
       </c>
       <c r="M58" s="5" t="s">
-        <v>339</v>
+        <v>89</v>
       </c>
       <c r="N58" s="5" t="s">
-        <v>396</v>
+        <v>373</v>
       </c>
       <c r="O58" s="5" t="s">
-        <v>397</v>
+        <v>374</v>
       </c>
       <c r="P58" s="6" t="s">
-        <v>398</v>
-      </c>
-      <c r="Q58" s="5" t="s">
-        <v>102</v>
-      </c>
+        <v>375</v>
+      </c>
+      <c r="Q58" s="5"/>
       <c r="R58" s="5"/>
     </row>
     <row r="59" spans="1:18" ht="18" customHeight="1">
@@ -5440,45 +5714,45 @@
         <v>22</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>391</v>
+        <v>376</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>399</v>
+        <v>377</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>400</v>
+        <v>378</v>
       </c>
       <c r="E59" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F59" s="5" t="s">
-        <v>401</v>
+        <v>379</v>
       </c>
       <c r="G59" s="6" t="s">
-        <v>402</v>
+        <v>380</v>
       </c>
       <c r="H59" s="9"/>
       <c r="I59" s="9"/>
       <c r="J59" s="5" t="s">
-        <v>28</v>
+        <v>98</v>
       </c>
       <c r="K59" s="5" t="s">
-        <v>39</v>
+        <v>78</v>
       </c>
       <c r="L59" s="5" t="s">
         <v>50</v>
       </c>
       <c r="M59" s="5" t="s">
-        <v>339</v>
+        <v>31</v>
       </c>
       <c r="N59" s="5" t="s">
-        <v>109</v>
+        <v>79</v>
       </c>
       <c r="O59" s="5" t="s">
-        <v>403</v>
+        <v>381</v>
       </c>
       <c r="P59" s="6" t="s">
-        <v>404</v>
+        <v>382</v>
       </c>
       <c r="Q59" s="5" t="s">
         <v>102</v>
@@ -5487,52 +5761,50 @@
     </row>
     <row r="60" spans="1:18" ht="18" customHeight="1">
       <c r="A60" s="5" t="s">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>405</v>
+        <v>376</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>406</v>
+        <v>383</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>407</v>
+        <v>384</v>
       </c>
       <c r="E60" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F60" s="5" t="s">
-        <v>408</v>
+        <v>86</v>
       </c>
       <c r="G60" s="6" t="s">
-        <v>409</v>
+        <v>385</v>
       </c>
       <c r="H60" s="9"/>
       <c r="I60" s="9"/>
       <c r="J60" s="5" t="s">
-        <v>28</v>
+        <v>204</v>
       </c>
       <c r="K60" s="5" t="s">
-        <v>39</v>
+        <v>78</v>
       </c>
       <c r="L60" s="5" t="s">
         <v>30</v>
       </c>
       <c r="M60" s="5" t="s">
-        <v>40</v>
+        <v>89</v>
       </c>
       <c r="N60" s="5" t="s">
-        <v>32</v>
+        <v>90</v>
       </c>
       <c r="O60" s="5" t="s">
-        <v>410</v>
+        <v>386</v>
       </c>
       <c r="P60" s="6" t="s">
-        <v>411</v>
-      </c>
-      <c r="Q60" s="5" t="s">
-        <v>102</v>
-      </c>
+        <v>387</v>
+      </c>
+      <c r="Q60" s="5"/>
       <c r="R60" s="5"/>
     </row>
     <row r="61" spans="1:18" ht="18" customHeight="1">
@@ -5540,95 +5812,99 @@
         <v>22</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>412</v>
+        <v>388</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>413</v>
+        <v>389</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>414</v>
+        <v>390</v>
       </c>
       <c r="E61" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F61" s="5" t="s">
-        <v>415</v>
+        <v>391</v>
       </c>
       <c r="G61" s="6" t="s">
-        <v>416</v>
+        <v>392</v>
       </c>
       <c r="H61" s="9"/>
       <c r="I61" s="9"/>
       <c r="J61" s="5" t="s">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="K61" s="5" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="L61" s="5" t="s">
-        <v>132</v>
+        <v>329</v>
       </c>
       <c r="M61" s="5" t="s">
-        <v>417</v>
+        <v>336</v>
       </c>
       <c r="N61" s="5" t="s">
-        <v>418</v>
+        <v>393</v>
       </c>
       <c r="O61" s="5" t="s">
-        <v>419</v>
+        <v>394</v>
       </c>
       <c r="P61" s="6" t="s">
-        <v>420</v>
-      </c>
-      <c r="Q61" s="5"/>
+        <v>395</v>
+      </c>
+      <c r="Q61" s="5" t="s">
+        <v>102</v>
+      </c>
       <c r="R61" s="5"/>
     </row>
     <row r="62" spans="1:18" ht="18" customHeight="1">
       <c r="A62" s="5" t="s">
-        <v>67</v>
+        <v>22</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>421</v>
+        <v>388</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>422</v>
+        <v>396</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>423</v>
+        <v>397</v>
       </c>
       <c r="E62" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F62" s="5" t="s">
-        <v>424</v>
+        <v>398</v>
       </c>
       <c r="G62" s="6" t="s">
-        <v>425</v>
+        <v>399</v>
       </c>
       <c r="H62" s="9"/>
       <c r="I62" s="9"/>
       <c r="J62" s="5" t="s">
-        <v>204</v>
+        <v>28</v>
       </c>
       <c r="K62" s="5" t="s">
-        <v>78</v>
+        <v>39</v>
       </c>
       <c r="L62" s="5" t="s">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="M62" s="5" t="s">
-        <v>89</v>
+        <v>336</v>
       </c>
       <c r="N62" s="5" t="s">
-        <v>58</v>
+        <v>109</v>
       </c>
       <c r="O62" s="5" t="s">
-        <v>426</v>
+        <v>400</v>
       </c>
       <c r="P62" s="6" t="s">
-        <v>427</v>
-      </c>
-      <c r="Q62" s="5"/>
+        <v>401</v>
+      </c>
+      <c r="Q62" s="5" t="s">
+        <v>102</v>
+      </c>
       <c r="R62" s="5"/>
     </row>
     <row r="63" spans="1:18" ht="18" customHeight="1">
@@ -5636,131 +5912,125 @@
         <v>22</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>421</v>
+        <v>402</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>428</v>
+        <v>403</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>429</v>
+        <v>404</v>
       </c>
       <c r="E63" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F63" s="5" t="s">
-        <v>157</v>
+        <v>405</v>
       </c>
       <c r="G63" s="6" t="s">
-        <v>430</v>
+        <v>406</v>
       </c>
       <c r="H63" s="9"/>
       <c r="I63" s="9"/>
       <c r="J63" s="5" t="s">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="K63" s="5" t="s">
-        <v>78</v>
+        <v>39</v>
       </c>
       <c r="L63" s="5" t="s">
         <v>30</v>
       </c>
       <c r="M63" s="5" t="s">
-        <v>89</v>
+        <v>40</v>
       </c>
       <c r="N63" s="5" t="s">
-        <v>109</v>
+        <v>32</v>
       </c>
       <c r="O63" s="5" t="s">
-        <v>431</v>
+        <v>407</v>
       </c>
       <c r="P63" s="6" t="s">
-        <v>432</v>
-      </c>
-      <c r="Q63" s="5"/>
+        <v>408</v>
+      </c>
+      <c r="Q63" s="5" t="s">
+        <v>102</v>
+      </c>
       <c r="R63" s="5"/>
     </row>
     <row r="64" spans="1:18" ht="18" customHeight="1">
       <c r="A64" s="5" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>342</v>
+        <v>409</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="D64" s="5" t="s">
-        <v>434</v>
+        <v>411</v>
       </c>
       <c r="E64" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F64" s="5" t="s">
-        <v>435</v>
+        <v>412</v>
       </c>
       <c r="G64" s="6" t="s">
-        <v>436</v>
-      </c>
-      <c r="H64" s="15">
-        <v>199.99</v>
-      </c>
-      <c r="I64" s="15" t="s">
-        <v>647</v>
-      </c>
+        <v>413</v>
+      </c>
+      <c r="H64" s="9"/>
+      <c r="I64" s="9"/>
       <c r="J64" s="5" t="s">
-        <v>204</v>
+        <v>48</v>
       </c>
       <c r="K64" s="5" t="s">
-        <v>78</v>
+        <v>49</v>
       </c>
       <c r="L64" s="5" t="s">
-        <v>30</v>
+        <v>132</v>
       </c>
       <c r="M64" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="N64" s="5"/>
+        <v>414</v>
+      </c>
+      <c r="N64" s="5" t="s">
+        <v>415</v>
+      </c>
       <c r="O64" s="5" t="s">
-        <v>437</v>
+        <v>416</v>
       </c>
       <c r="P64" s="6" t="s">
-        <v>438</v>
-      </c>
-      <c r="Q64" s="8" t="s">
-        <v>439</v>
-      </c>
+        <v>417</v>
+      </c>
+      <c r="Q64" s="5"/>
       <c r="R64" s="5"/>
     </row>
     <row r="65" spans="1:18" ht="18" customHeight="1">
       <c r="A65" s="5" t="s">
-        <v>44</v>
+        <v>67</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>342</v>
+        <v>418</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>440</v>
+        <v>419</v>
       </c>
       <c r="D65" s="5" t="s">
-        <v>441</v>
+        <v>420</v>
       </c>
       <c r="E65" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F65" s="5" t="s">
-        <v>442</v>
+        <v>421</v>
       </c>
       <c r="G65" s="6" t="s">
-        <v>443</v>
-      </c>
-      <c r="H65" s="15">
-        <v>299.99</v>
-      </c>
-      <c r="I65" s="15" t="s">
-        <v>646</v>
-      </c>
+        <v>422</v>
+      </c>
+      <c r="H65" s="9"/>
+      <c r="I65" s="9"/>
       <c r="J65" s="5" t="s">
-        <v>48</v>
+        <v>204</v>
       </c>
       <c r="K65" s="5" t="s">
         <v>78</v>
@@ -5772,45 +6042,43 @@
         <v>89</v>
       </c>
       <c r="N65" s="5" t="s">
-        <v>444</v>
+        <v>58</v>
       </c>
       <c r="O65" s="5" t="s">
-        <v>445</v>
+        <v>423</v>
       </c>
       <c r="P65" s="6" t="s">
-        <v>446</v>
-      </c>
-      <c r="Q65" s="8" t="s">
-        <v>447</v>
-      </c>
+        <v>424</v>
+      </c>
+      <c r="Q65" s="5"/>
       <c r="R65" s="5"/>
     </row>
     <row r="66" spans="1:18" ht="18" customHeight="1">
       <c r="A66" s="5" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>150</v>
+        <v>418</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>448</v>
+        <v>425</v>
       </c>
       <c r="D66" s="5" t="s">
-        <v>449</v>
+        <v>426</v>
       </c>
       <c r="E66" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F66" s="5" t="s">
-        <v>450</v>
+        <v>157</v>
       </c>
       <c r="G66" s="6" t="s">
-        <v>146</v>
+        <v>427</v>
       </c>
       <c r="H66" s="9"/>
       <c r="I66" s="9"/>
       <c r="J66" s="5" t="s">
-        <v>98</v>
+        <v>48</v>
       </c>
       <c r="K66" s="5" t="s">
         <v>78</v>
@@ -5822,13 +6090,13 @@
         <v>89</v>
       </c>
       <c r="N66" s="5" t="s">
-        <v>369</v>
+        <v>109</v>
       </c>
       <c r="O66" s="5" t="s">
-        <v>451</v>
+        <v>428</v>
       </c>
       <c r="P66" s="6" t="s">
-        <v>452</v>
+        <v>429</v>
       </c>
       <c r="Q66" s="5"/>
       <c r="R66" s="5"/>
@@ -5838,31 +6106,31 @@
         <v>44</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>247</v>
+        <v>339</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>453</v>
+        <v>430</v>
       </c>
       <c r="D67" s="5" t="s">
-        <v>454</v>
+        <v>431</v>
       </c>
       <c r="E67" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F67" s="5" t="s">
-        <v>450</v>
+        <v>432</v>
       </c>
       <c r="G67" s="6" t="s">
-        <v>455</v>
-      </c>
-      <c r="H67" s="15">
-        <v>449.99</v>
-      </c>
-      <c r="I67" s="15" t="s">
-        <v>648</v>
+        <v>433</v>
+      </c>
+      <c r="H67" s="11">
+        <v>199.99</v>
+      </c>
+      <c r="I67" s="11" t="s">
+        <v>644</v>
       </c>
       <c r="J67" s="5" t="s">
-        <v>98</v>
+        <v>204</v>
       </c>
       <c r="K67" s="5" t="s">
         <v>78</v>
@@ -5873,50 +6141,48 @@
       <c r="M67" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="N67" s="5" t="s">
-        <v>369</v>
-      </c>
+      <c r="N67" s="5"/>
       <c r="O67" s="5" t="s">
-        <v>451</v>
+        <v>434</v>
       </c>
       <c r="P67" s="6" t="s">
-        <v>456</v>
+        <v>435</v>
       </c>
       <c r="Q67" s="8" t="s">
-        <v>457</v>
+        <v>436</v>
       </c>
       <c r="R67" s="5"/>
     </row>
     <row r="68" spans="1:18" ht="18" customHeight="1">
       <c r="A68" s="5" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="B68" s="5" t="s">
-        <v>247</v>
+        <v>339</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>458</v>
+        <v>437</v>
       </c>
       <c r="D68" s="5" t="s">
-        <v>459</v>
+        <v>438</v>
       </c>
       <c r="E68" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F68" s="5" t="s">
-        <v>460</v>
+        <v>439</v>
       </c>
       <c r="G68" s="6" t="s">
-        <v>461</v>
-      </c>
-      <c r="H68" s="15">
-        <v>679.99</v>
-      </c>
-      <c r="I68" s="15" t="s">
-        <v>649</v>
+        <v>440</v>
+      </c>
+      <c r="H68" s="11">
+        <v>299.99</v>
+      </c>
+      <c r="I68" s="11" t="s">
+        <v>643</v>
       </c>
       <c r="J68" s="5" t="s">
-        <v>98</v>
+        <v>48</v>
       </c>
       <c r="K68" s="5" t="s">
         <v>78</v>
@@ -5928,16 +6194,16 @@
         <v>89</v>
       </c>
       <c r="N68" s="5" t="s">
-        <v>109</v>
+        <v>441</v>
       </c>
       <c r="O68" s="5" t="s">
-        <v>462</v>
+        <v>442</v>
       </c>
       <c r="P68" s="6" t="s">
-        <v>463</v>
+        <v>443</v>
       </c>
       <c r="Q68" s="8" t="s">
-        <v>464</v>
+        <v>444</v>
       </c>
       <c r="R68" s="5"/>
     </row>
@@ -5946,29 +6212,25 @@
         <v>44</v>
       </c>
       <c r="B69" s="5" t="s">
-        <v>247</v>
+        <v>150</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>458</v>
+        <v>445</v>
       </c>
       <c r="D69" s="5" t="s">
-        <v>465</v>
+        <v>446</v>
       </c>
       <c r="E69" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F69" s="5" t="s">
-        <v>460</v>
+        <v>447</v>
       </c>
       <c r="G69" s="6" t="s">
-        <v>466</v>
-      </c>
-      <c r="H69" s="15">
-        <v>679.99</v>
-      </c>
-      <c r="I69" s="15" t="s">
-        <v>650</v>
-      </c>
+        <v>146</v>
+      </c>
+      <c r="H69" s="9"/>
+      <c r="I69" s="9"/>
       <c r="J69" s="5" t="s">
         <v>98</v>
       </c>
@@ -5982,17 +6244,15 @@
         <v>89</v>
       </c>
       <c r="N69" s="5" t="s">
-        <v>109</v>
+        <v>366</v>
       </c>
       <c r="O69" s="5" t="s">
-        <v>462</v>
+        <v>448</v>
       </c>
       <c r="P69" s="6" t="s">
-        <v>467</v>
-      </c>
-      <c r="Q69" s="8" t="s">
-        <v>468</v>
-      </c>
+        <v>449</v>
+      </c>
+      <c r="Q69" s="5"/>
       <c r="R69" s="5"/>
     </row>
     <row r="70" spans="1:18" ht="18" customHeight="1">
@@ -6000,30 +6260,34 @@
         <v>44</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>93</v>
+        <v>247</v>
       </c>
       <c r="C70" s="5" t="s">
-        <v>469</v>
+        <v>450</v>
       </c>
       <c r="D70" s="5" t="s">
-        <v>470</v>
+        <v>451</v>
       </c>
       <c r="E70" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F70" s="5" t="s">
-        <v>471</v>
+        <v>447</v>
       </c>
       <c r="G70" s="6" t="s">
-        <v>472</v>
-      </c>
-      <c r="H70" s="9"/>
-      <c r="I70" s="9"/>
+        <v>452</v>
+      </c>
+      <c r="H70" s="11">
+        <v>449.99</v>
+      </c>
+      <c r="I70" s="11" t="s">
+        <v>645</v>
+      </c>
       <c r="J70" s="5" t="s">
-        <v>28</v>
+        <v>98</v>
       </c>
       <c r="K70" s="5" t="s">
-        <v>39</v>
+        <v>78</v>
       </c>
       <c r="L70" s="5" t="s">
         <v>30</v>
@@ -6032,43 +6296,49 @@
         <v>89</v>
       </c>
       <c r="N70" s="5" t="s">
-        <v>473</v>
+        <v>366</v>
       </c>
       <c r="O70" s="5" t="s">
-        <v>474</v>
+        <v>448</v>
       </c>
       <c r="P70" s="6" t="s">
-        <v>475</v>
-      </c>
-      <c r="Q70" s="5"/>
+        <v>453</v>
+      </c>
+      <c r="Q70" s="8" t="s">
+        <v>454</v>
+      </c>
       <c r="R70" s="5"/>
     </row>
     <row r="71" spans="1:18" ht="18" customHeight="1">
       <c r="A71" s="5" t="s">
-        <v>44</v>
+        <v>67</v>
       </c>
       <c r="B71" s="5" t="s">
         <v>247</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>476</v>
+        <v>455</v>
       </c>
       <c r="D71" s="5" t="s">
-        <v>477</v>
+        <v>456</v>
       </c>
       <c r="E71" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F71" s="5" t="s">
-        <v>478</v>
+        <v>457</v>
       </c>
       <c r="G71" s="6" t="s">
-        <v>479</v>
-      </c>
-      <c r="H71" s="9"/>
-      <c r="I71" s="9"/>
+        <v>458</v>
+      </c>
+      <c r="H71" s="11">
+        <v>679.99</v>
+      </c>
+      <c r="I71" s="11" t="s">
+        <v>646</v>
+      </c>
       <c r="J71" s="5" t="s">
-        <v>28</v>
+        <v>98</v>
       </c>
       <c r="K71" s="5" t="s">
         <v>78</v>
@@ -6080,15 +6350,17 @@
         <v>89</v>
       </c>
       <c r="N71" s="5" t="s">
-        <v>58</v>
+        <v>109</v>
       </c>
       <c r="O71" s="5" t="s">
-        <v>480</v>
+        <v>459</v>
       </c>
       <c r="P71" s="6" t="s">
-        <v>481</v>
-      </c>
-      <c r="Q71" s="5"/>
+        <v>460</v>
+      </c>
+      <c r="Q71" s="8" t="s">
+        <v>461</v>
+      </c>
       <c r="R71" s="5"/>
     </row>
     <row r="72" spans="1:18" ht="18" customHeight="1">
@@ -6096,27 +6368,31 @@
         <v>44</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>342</v>
+        <v>247</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>482</v>
+        <v>455</v>
       </c>
       <c r="D72" s="5" t="s">
-        <v>483</v>
+        <v>462</v>
       </c>
       <c r="E72" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F72" s="5" t="s">
-        <v>484</v>
+        <v>457</v>
       </c>
       <c r="G72" s="6" t="s">
-        <v>485</v>
-      </c>
-      <c r="H72" s="9"/>
-      <c r="I72" s="9"/>
+        <v>463</v>
+      </c>
+      <c r="H72" s="11">
+        <v>679.99</v>
+      </c>
+      <c r="I72" s="11" t="s">
+        <v>647</v>
+      </c>
       <c r="J72" s="5" t="s">
-        <v>204</v>
+        <v>98</v>
       </c>
       <c r="K72" s="5" t="s">
         <v>78</v>
@@ -6128,15 +6404,17 @@
         <v>89</v>
       </c>
       <c r="N72" s="5" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="O72" s="5" t="s">
-        <v>486</v>
+        <v>459</v>
       </c>
       <c r="P72" s="6" t="s">
-        <v>487</v>
-      </c>
-      <c r="Q72" s="5"/>
+        <v>464</v>
+      </c>
+      <c r="Q72" s="8" t="s">
+        <v>465</v>
+      </c>
       <c r="R72" s="5"/>
     </row>
     <row r="73" spans="1:18" ht="18" customHeight="1">
@@ -6144,53 +6422,47 @@
         <v>44</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>247</v>
+        <v>93</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>488</v>
+        <v>466</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>489</v>
+        <v>467</v>
       </c>
       <c r="E73" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F73" s="5" t="s">
-        <v>490</v>
+        <v>468</v>
       </c>
       <c r="G73" s="6" t="s">
-        <v>491</v>
-      </c>
-      <c r="H73" s="15">
-        <v>379.99</v>
-      </c>
-      <c r="I73" s="15" t="s">
-        <v>651</v>
-      </c>
+        <v>469</v>
+      </c>
+      <c r="H73" s="9"/>
+      <c r="I73" s="9"/>
       <c r="J73" s="5" t="s">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="K73" s="5" t="s">
-        <v>78</v>
+        <v>39</v>
       </c>
       <c r="L73" s="5" t="s">
-        <v>132</v>
+        <v>30</v>
       </c>
       <c r="M73" s="5" t="s">
         <v>89</v>
       </c>
       <c r="N73" s="5" t="s">
-        <v>205</v>
+        <v>470</v>
       </c>
       <c r="O73" s="5" t="s">
-        <v>492</v>
+        <v>471</v>
       </c>
       <c r="P73" s="6" t="s">
-        <v>493</v>
-      </c>
-      <c r="Q73" s="20" t="s">
-        <v>652</v>
-      </c>
+        <v>472</v>
+      </c>
+      <c r="Q73" s="5"/>
       <c r="R73" s="5"/>
     </row>
     <row r="74" spans="1:18" ht="18" customHeight="1">
@@ -6201,28 +6473,24 @@
         <v>247</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>494</v>
+        <v>473</v>
       </c>
       <c r="D74" s="5" t="s">
-        <v>495</v>
+        <v>474</v>
       </c>
       <c r="E74" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F74" s="5" t="s">
-        <v>496</v>
-      </c>
-      <c r="G74" s="17">
-        <v>299.99</v>
-      </c>
-      <c r="H74" s="15">
-        <v>299.99</v>
-      </c>
-      <c r="I74" s="15" t="s">
-        <v>658</v>
-      </c>
+        <v>475</v>
+      </c>
+      <c r="G74" s="6" t="s">
+        <v>476</v>
+      </c>
+      <c r="H74" s="9"/>
+      <c r="I74" s="9"/>
       <c r="J74" s="5" t="s">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="K74" s="5" t="s">
         <v>78</v>
@@ -6234,17 +6502,15 @@
         <v>89</v>
       </c>
       <c r="N74" s="5" t="s">
-        <v>99</v>
+        <v>58</v>
       </c>
       <c r="O74" s="5" t="s">
-        <v>497</v>
+        <v>477</v>
       </c>
       <c r="P74" s="6" t="s">
-        <v>498</v>
-      </c>
-      <c r="Q74" s="20" t="s">
-        <v>653</v>
-      </c>
+        <v>478</v>
+      </c>
+      <c r="Q74" s="5"/>
       <c r="R74" s="5"/>
     </row>
     <row r="75" spans="1:18" ht="18" customHeight="1">
@@ -6252,82 +6518,76 @@
         <v>44</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>247</v>
+        <v>339</v>
       </c>
       <c r="C75" s="5" t="s">
-        <v>499</v>
+        <v>479</v>
       </c>
       <c r="D75" s="5" t="s">
-        <v>500</v>
+        <v>480</v>
       </c>
       <c r="E75" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F75" s="5" t="s">
-        <v>501</v>
+        <v>481</v>
       </c>
       <c r="G75" s="6" t="s">
-        <v>502</v>
-      </c>
-      <c r="H75" s="15">
-        <v>1299.99</v>
-      </c>
-      <c r="I75" s="15" t="s">
-        <v>657</v>
-      </c>
+        <v>482</v>
+      </c>
+      <c r="H75" s="9"/>
+      <c r="I75" s="9"/>
       <c r="J75" s="5" t="s">
-        <v>28</v>
+        <v>204</v>
       </c>
       <c r="K75" s="5" t="s">
-        <v>39</v>
+        <v>78</v>
       </c>
       <c r="L75" s="5" t="s">
         <v>30</v>
       </c>
       <c r="M75" s="5" t="s">
-        <v>503</v>
+        <v>89</v>
       </c>
       <c r="N75" s="5" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="O75" s="5" t="s">
-        <v>504</v>
+        <v>483</v>
       </c>
       <c r="P75" s="6" t="s">
-        <v>505</v>
-      </c>
-      <c r="Q75" s="8" t="s">
-        <v>506</v>
-      </c>
+        <v>484</v>
+      </c>
+      <c r="Q75" s="5"/>
       <c r="R75" s="5"/>
     </row>
     <row r="76" spans="1:18" ht="18" customHeight="1">
       <c r="A76" s="5" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="B76" s="5" t="s">
         <v>247</v>
       </c>
       <c r="C76" s="5" t="s">
-        <v>507</v>
+        <v>485</v>
       </c>
       <c r="D76" s="5" t="s">
-        <v>508</v>
+        <v>486</v>
       </c>
       <c r="E76" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F76" s="5" t="s">
-        <v>509</v>
+        <v>487</v>
       </c>
       <c r="G76" s="6" t="s">
-        <v>158</v>
-      </c>
-      <c r="H76" s="15">
-        <v>399.99</v>
-      </c>
-      <c r="I76" s="15" t="s">
-        <v>654</v>
+        <v>488</v>
+      </c>
+      <c r="H76" s="11">
+        <v>379.99</v>
+      </c>
+      <c r="I76" s="11" t="s">
+        <v>648</v>
       </c>
       <c r="J76" s="5" t="s">
         <v>48</v>
@@ -6336,109 +6596,109 @@
         <v>78</v>
       </c>
       <c r="L76" s="5" t="s">
-        <v>30</v>
+        <v>132</v>
       </c>
       <c r="M76" s="5" t="s">
-        <v>503</v>
+        <v>89</v>
       </c>
       <c r="N76" s="5" t="s">
-        <v>369</v>
+        <v>205</v>
       </c>
       <c r="O76" s="5" t="s">
-        <v>510</v>
+        <v>489</v>
       </c>
       <c r="P76" s="6" t="s">
-        <v>511</v>
-      </c>
-      <c r="Q76" s="8" t="s">
-        <v>512</v>
+        <v>490</v>
+      </c>
+      <c r="Q76" s="16" t="s">
+        <v>649</v>
       </c>
       <c r="R76" s="5"/>
     </row>
     <row r="77" spans="1:18" ht="18" customHeight="1">
       <c r="A77" s="5" t="s">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="B77" s="5" t="s">
         <v>247</v>
       </c>
       <c r="C77" s="5" t="s">
-        <v>513</v>
+        <v>491</v>
       </c>
       <c r="D77" s="5" t="s">
-        <v>514</v>
+        <v>492</v>
       </c>
       <c r="E77" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F77" s="5" t="s">
-        <v>515</v>
-      </c>
-      <c r="G77" s="6" t="s">
-        <v>461</v>
-      </c>
-      <c r="H77" s="15">
-        <v>699.99</v>
-      </c>
-      <c r="I77" s="15" t="s">
-        <v>656</v>
+        <v>493</v>
+      </c>
+      <c r="G77" s="13">
+        <v>299.99</v>
+      </c>
+      <c r="H77" s="11">
+        <v>299.99</v>
+      </c>
+      <c r="I77" s="11" t="s">
+        <v>655</v>
       </c>
       <c r="J77" s="5" t="s">
-        <v>98</v>
+        <v>48</v>
       </c>
       <c r="K77" s="5" t="s">
-        <v>39</v>
+        <v>78</v>
       </c>
       <c r="L77" s="5" t="s">
         <v>30</v>
       </c>
       <c r="M77" s="5" t="s">
-        <v>516</v>
+        <v>89</v>
       </c>
       <c r="N77" s="5" t="s">
-        <v>517</v>
+        <v>99</v>
       </c>
       <c r="O77" s="5" t="s">
-        <v>518</v>
+        <v>494</v>
       </c>
       <c r="P77" s="6" t="s">
-        <v>519</v>
-      </c>
-      <c r="Q77" s="8" t="s">
-        <v>520</v>
+        <v>495</v>
+      </c>
+      <c r="Q77" s="16" t="s">
+        <v>650</v>
       </c>
       <c r="R77" s="5"/>
     </row>
     <row r="78" spans="1:18" ht="18" customHeight="1">
       <c r="A78" s="5" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="B78" s="5" t="s">
         <v>247</v>
       </c>
       <c r="C78" s="5" t="s">
-        <v>513</v>
+        <v>496</v>
       </c>
       <c r="D78" s="5" t="s">
-        <v>521</v>
+        <v>497</v>
       </c>
       <c r="E78" s="5" t="s">
         <v>26</v>
       </c>
       <c r="F78" s="5" t="s">
-        <v>522</v>
+        <v>498</v>
       </c>
       <c r="G78" s="6" t="s">
-        <v>461</v>
-      </c>
-      <c r="H78" s="15">
-        <v>699.99</v>
-      </c>
-      <c r="I78" s="15" t="s">
-        <v>659</v>
+        <v>499</v>
+      </c>
+      <c r="H78" s="11">
+        <v>1299.99</v>
+      </c>
+      <c r="I78" s="11" t="s">
+        <v>654</v>
       </c>
       <c r="J78" s="5" t="s">
-        <v>98</v>
+        <v>28</v>
       </c>
       <c r="K78" s="5" t="s">
         <v>39</v>
@@ -6447,120 +6707,128 @@
         <v>30</v>
       </c>
       <c r="M78" s="5" t="s">
-        <v>516</v>
+        <v>500</v>
       </c>
       <c r="N78" s="5" t="s">
-        <v>517</v>
+        <v>109</v>
       </c>
       <c r="O78" s="5" t="s">
-        <v>523</v>
+        <v>501</v>
       </c>
       <c r="P78" s="6" t="s">
-        <v>524</v>
+        <v>502</v>
       </c>
       <c r="Q78" s="8" t="s">
-        <v>525</v>
+        <v>503</v>
       </c>
       <c r="R78" s="5"/>
     </row>
     <row r="79" spans="1:18" ht="18" customHeight="1">
       <c r="A79" s="5" t="s">
-        <v>22</v>
+        <v>67</v>
       </c>
       <c r="B79" s="5" t="s">
-        <v>526</v>
+        <v>247</v>
       </c>
       <c r="C79" s="5" t="s">
-        <v>527</v>
+        <v>504</v>
       </c>
       <c r="D79" s="5" t="s">
-        <v>528</v>
+        <v>505</v>
       </c>
       <c r="E79" s="5" t="s">
-        <v>529</v>
+        <v>26</v>
       </c>
       <c r="F79" s="5" t="s">
-        <v>530</v>
+        <v>506</v>
       </c>
       <c r="G79" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="H79" s="9"/>
-      <c r="I79" s="9"/>
+        <v>158</v>
+      </c>
+      <c r="H79" s="11">
+        <v>399.99</v>
+      </c>
+      <c r="I79" s="11" t="s">
+        <v>651</v>
+      </c>
       <c r="J79" s="5" t="s">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="K79" s="5" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="L79" s="5" t="s">
         <v>30</v>
       </c>
       <c r="M79" s="5" t="s">
-        <v>531</v>
+        <v>500</v>
       </c>
       <c r="N79" s="5" t="s">
-        <v>109</v>
+        <v>366</v>
       </c>
       <c r="O79" s="5" t="s">
-        <v>532</v>
+        <v>507</v>
       </c>
       <c r="P79" s="6" t="s">
-        <v>533</v>
-      </c>
-      <c r="Q79" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="R79" s="5" t="s">
-        <v>534</v>
-      </c>
+        <v>508</v>
+      </c>
+      <c r="Q79" s="8" t="s">
+        <v>509</v>
+      </c>
+      <c r="R79" s="5"/>
     </row>
     <row r="80" spans="1:18" ht="18" customHeight="1">
       <c r="A80" s="5" t="s">
-        <v>67</v>
+        <v>22</v>
       </c>
       <c r="B80" s="5" t="s">
-        <v>526</v>
+        <v>247</v>
       </c>
       <c r="C80" s="5" t="s">
-        <v>527</v>
+        <v>510</v>
       </c>
       <c r="D80" s="5" t="s">
-        <v>535</v>
+        <v>511</v>
       </c>
       <c r="E80" s="5" t="s">
-        <v>529</v>
+        <v>26</v>
       </c>
       <c r="F80" s="5" t="s">
-        <v>530</v>
+        <v>512</v>
       </c>
       <c r="G80" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="H80" s="9"/>
-      <c r="I80" s="9"/>
+        <v>458</v>
+      </c>
+      <c r="H80" s="11">
+        <v>699.99</v>
+      </c>
+      <c r="I80" s="11" t="s">
+        <v>653</v>
+      </c>
       <c r="J80" s="5" t="s">
-        <v>28</v>
+        <v>98</v>
       </c>
       <c r="K80" s="5" t="s">
-        <v>88</v>
+        <v>39</v>
       </c>
       <c r="L80" s="5" t="s">
         <v>30</v>
       </c>
       <c r="M80" s="5" t="s">
-        <v>531</v>
+        <v>513</v>
       </c>
       <c r="N80" s="5" t="s">
-        <v>109</v>
+        <v>514</v>
       </c>
       <c r="O80" s="5" t="s">
-        <v>532</v>
+        <v>515</v>
       </c>
       <c r="P80" s="6" t="s">
-        <v>536</v>
-      </c>
-      <c r="Q80" s="5"/>
+        <v>516</v>
+      </c>
+      <c r="Q80" s="8" t="s">
+        <v>517</v>
+      </c>
       <c r="R80" s="5"/>
     </row>
     <row r="81" spans="1:18" ht="18" customHeight="1">
@@ -6568,27 +6836,31 @@
         <v>67</v>
       </c>
       <c r="B81" s="5" t="s">
-        <v>526</v>
+        <v>247</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>537</v>
+        <v>510</v>
       </c>
       <c r="D81" s="5" t="s">
-        <v>538</v>
+        <v>518</v>
       </c>
       <c r="E81" s="5" t="s">
-        <v>539</v>
+        <v>26</v>
       </c>
       <c r="F81" s="5" t="s">
-        <v>540</v>
+        <v>519</v>
       </c>
       <c r="G81" s="6" t="s">
-        <v>541</v>
-      </c>
-      <c r="H81" s="9"/>
-      <c r="I81" s="9"/>
+        <v>458</v>
+      </c>
+      <c r="H81" s="11">
+        <v>699.99</v>
+      </c>
+      <c r="I81" s="11" t="s">
+        <v>656</v>
+      </c>
       <c r="J81" s="5" t="s">
-        <v>28</v>
+        <v>98</v>
       </c>
       <c r="K81" s="5" t="s">
         <v>39</v>
@@ -6597,48 +6869,46 @@
         <v>30</v>
       </c>
       <c r="M81" s="5" t="s">
-        <v>531</v>
+        <v>513</v>
       </c>
       <c r="N81" s="5" t="s">
-        <v>473</v>
+        <v>514</v>
       </c>
       <c r="O81" s="5" t="s">
-        <v>542</v>
+        <v>520</v>
       </c>
       <c r="P81" s="6" t="s">
-        <v>543</v>
-      </c>
-      <c r="Q81" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="R81" s="5" t="s">
-        <v>534</v>
-      </c>
+        <v>521</v>
+      </c>
+      <c r="Q81" s="8" t="s">
+        <v>522</v>
+      </c>
+      <c r="R81" s="5"/>
     </row>
     <row r="82" spans="1:18" ht="18" customHeight="1">
       <c r="A82" s="5" t="s">
         <v>22</v>
       </c>
       <c r="B82" s="5" t="s">
+        <v>523</v>
+      </c>
+      <c r="C82" s="5" t="s">
+        <v>524</v>
+      </c>
+      <c r="D82" s="5" t="s">
+        <v>525</v>
+      </c>
+      <c r="E82" s="5" t="s">
         <v>526</v>
       </c>
-      <c r="C82" s="5" t="s">
-        <v>544</v>
-      </c>
-      <c r="D82" s="5" t="s">
-        <v>545</v>
-      </c>
-      <c r="E82" s="5" t="s">
-        <v>546</v>
-      </c>
       <c r="F82" s="5" t="s">
-        <v>547</v>
+        <v>527</v>
       </c>
       <c r="G82" s="6" t="s">
-        <v>548</v>
-      </c>
-      <c r="H82" s="7"/>
-      <c r="I82" s="7"/>
+        <v>238</v>
+      </c>
+      <c r="H82" s="9"/>
+      <c r="I82" s="9"/>
       <c r="J82" s="5" t="s">
         <v>28</v>
       </c>
@@ -6646,25 +6916,25 @@
         <v>88</v>
       </c>
       <c r="L82" s="5" t="s">
-        <v>132</v>
+        <v>30</v>
       </c>
       <c r="M82" s="5" t="s">
-        <v>339</v>
+        <v>528</v>
       </c>
       <c r="N82" s="5" t="s">
         <v>109</v>
       </c>
       <c r="O82" s="5" t="s">
-        <v>549</v>
+        <v>529</v>
       </c>
       <c r="P82" s="6" t="s">
-        <v>550</v>
-      </c>
-      <c r="Q82" s="8" t="s">
-        <v>551</v>
+        <v>530</v>
+      </c>
+      <c r="Q82" s="5" t="s">
+        <v>102</v>
       </c>
       <c r="R82" s="5" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
     </row>
     <row r="83" spans="1:18" ht="18" customHeight="1">
@@ -6672,74 +6942,70 @@
         <v>67</v>
       </c>
       <c r="B83" s="5" t="s">
+        <v>523</v>
+      </c>
+      <c r="C83" s="5" t="s">
+        <v>524</v>
+      </c>
+      <c r="D83" s="5" t="s">
+        <v>532</v>
+      </c>
+      <c r="E83" s="5" t="s">
         <v>526</v>
       </c>
-      <c r="C83" s="5" t="s">
-        <v>552</v>
-      </c>
-      <c r="D83" s="5" t="s">
-        <v>553</v>
-      </c>
-      <c r="E83" s="5" t="s">
-        <v>554</v>
-      </c>
       <c r="F83" s="5" t="s">
-        <v>555</v>
+        <v>527</v>
       </c>
       <c r="G83" s="6" t="s">
-        <v>556</v>
+        <v>120</v>
       </c>
       <c r="H83" s="9"/>
       <c r="I83" s="9"/>
       <c r="J83" s="5" t="s">
-        <v>98</v>
+        <v>28</v>
       </c>
       <c r="K83" s="5" t="s">
-        <v>39</v>
+        <v>88</v>
       </c>
       <c r="L83" s="5" t="s">
         <v>30</v>
       </c>
       <c r="M83" s="5" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="N83" s="5" t="s">
-        <v>473</v>
+        <v>109</v>
       </c>
       <c r="O83" s="5" t="s">
-        <v>557</v>
+        <v>529</v>
       </c>
       <c r="P83" s="6" t="s">
-        <v>558</v>
-      </c>
-      <c r="Q83" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="R83" s="5" t="s">
-        <v>534</v>
-      </c>
+        <v>533</v>
+      </c>
+      <c r="Q83" s="5"/>
+      <c r="R83" s="5"/>
     </row>
     <row r="84" spans="1:18" ht="18" customHeight="1">
       <c r="A84" s="5" t="s">
-        <v>22</v>
+        <v>67</v>
       </c>
       <c r="B84" s="5" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>552</v>
+        <v>534</v>
       </c>
       <c r="D84" s="5" t="s">
-        <v>559</v>
+        <v>535</v>
       </c>
       <c r="E84" s="5" t="s">
-        <v>554</v>
+        <v>536</v>
       </c>
       <c r="F84" s="5" t="s">
-        <v>555</v>
+        <v>537</v>
       </c>
       <c r="G84" s="6" t="s">
-        <v>560</v>
+        <v>538</v>
       </c>
       <c r="H84" s="9"/>
       <c r="I84" s="9"/>
@@ -6753,44 +7019,48 @@
         <v>30</v>
       </c>
       <c r="M84" s="5" t="s">
+        <v>528</v>
+      </c>
+      <c r="N84" s="5" t="s">
+        <v>470</v>
+      </c>
+      <c r="O84" s="5" t="s">
+        <v>539</v>
+      </c>
+      <c r="P84" s="6" t="s">
+        <v>540</v>
+      </c>
+      <c r="Q84" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="R84" s="5" t="s">
         <v>531</v>
       </c>
-      <c r="N84" s="5" t="s">
-        <v>473</v>
-      </c>
-      <c r="O84" s="5" t="s">
-        <v>557</v>
-      </c>
-      <c r="P84" s="6" t="s">
-        <v>561</v>
-      </c>
-      <c r="Q84" s="5"/>
-      <c r="R84" s="5"/>
     </row>
     <row r="85" spans="1:18" ht="18" customHeight="1">
       <c r="A85" s="5" t="s">
         <v>22</v>
       </c>
       <c r="B85" s="5" t="s">
-        <v>562</v>
+        <v>523</v>
       </c>
       <c r="C85" s="5" t="s">
-        <v>563</v>
+        <v>541</v>
       </c>
       <c r="D85" s="5" t="s">
-        <v>564</v>
+        <v>542</v>
       </c>
       <c r="E85" s="5" t="s">
-        <v>565</v>
+        <v>543</v>
       </c>
       <c r="F85" s="5" t="s">
-        <v>566</v>
+        <v>544</v>
       </c>
       <c r="G85" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="H85" s="9"/>
-      <c r="I85" s="9"/>
+        <v>545</v>
+      </c>
+      <c r="H85" s="7"/>
+      <c r="I85" s="7"/>
       <c r="J85" s="5" t="s">
         <v>28</v>
       </c>
@@ -6798,25 +7068,25 @@
         <v>88</v>
       </c>
       <c r="L85" s="5" t="s">
-        <v>30</v>
+        <v>132</v>
       </c>
       <c r="M85" s="5" t="s">
-        <v>531</v>
+        <v>336</v>
       </c>
       <c r="N85" s="5" t="s">
         <v>109</v>
       </c>
       <c r="O85" s="5" t="s">
-        <v>567</v>
+        <v>546</v>
       </c>
       <c r="P85" s="6" t="s">
-        <v>568</v>
-      </c>
-      <c r="Q85" s="5" t="s">
-        <v>102</v>
+        <v>547</v>
+      </c>
+      <c r="Q85" s="8" t="s">
+        <v>548</v>
       </c>
       <c r="R85" s="5" t="s">
-        <v>103</v>
+        <v>531</v>
       </c>
     </row>
     <row r="86" spans="1:18" ht="18" customHeight="1">
@@ -6824,70 +7094,74 @@
         <v>67</v>
       </c>
       <c r="B86" s="5" t="s">
-        <v>562</v>
+        <v>523</v>
       </c>
       <c r="C86" s="5" t="s">
-        <v>563</v>
+        <v>549</v>
       </c>
       <c r="D86" s="5" t="s">
-        <v>569</v>
+        <v>550</v>
       </c>
       <c r="E86" s="5" t="s">
-        <v>565</v>
+        <v>551</v>
       </c>
       <c r="F86" s="5" t="s">
-        <v>566</v>
+        <v>552</v>
       </c>
       <c r="G86" s="6" t="s">
-        <v>502</v>
+        <v>553</v>
       </c>
       <c r="H86" s="9"/>
       <c r="I86" s="9"/>
       <c r="J86" s="5" t="s">
-        <v>28</v>
+        <v>98</v>
       </c>
       <c r="K86" s="5" t="s">
-        <v>88</v>
+        <v>39</v>
       </c>
       <c r="L86" s="5" t="s">
         <v>30</v>
       </c>
       <c r="M86" s="5" t="s">
+        <v>528</v>
+      </c>
+      <c r="N86" s="5" t="s">
+        <v>470</v>
+      </c>
+      <c r="O86" s="5" t="s">
+        <v>554</v>
+      </c>
+      <c r="P86" s="6" t="s">
+        <v>555</v>
+      </c>
+      <c r="Q86" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="R86" s="5" t="s">
         <v>531</v>
       </c>
-      <c r="N86" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="O86" s="5" t="s">
-        <v>567</v>
-      </c>
-      <c r="P86" s="6" t="s">
-        <v>570</v>
-      </c>
-      <c r="Q86" s="5"/>
-      <c r="R86" s="5"/>
     </row>
     <row r="87" spans="1:18" ht="18" customHeight="1">
       <c r="A87" s="5" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="B87" s="5" t="s">
-        <v>562</v>
+        <v>523</v>
       </c>
       <c r="C87" s="5" t="s">
-        <v>571</v>
+        <v>549</v>
       </c>
       <c r="D87" s="5" t="s">
-        <v>572</v>
+        <v>556</v>
       </c>
       <c r="E87" s="5" t="s">
-        <v>573</v>
+        <v>551</v>
       </c>
       <c r="F87" s="5" t="s">
-        <v>574</v>
+        <v>552</v>
       </c>
       <c r="G87" s="6" t="s">
-        <v>575</v>
+        <v>557</v>
       </c>
       <c r="H87" s="9"/>
       <c r="I87" s="9"/>
@@ -6901,45 +7175,41 @@
         <v>30</v>
       </c>
       <c r="M87" s="5" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="N87" s="5" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="O87" s="5" t="s">
-        <v>576</v>
+        <v>554</v>
       </c>
       <c r="P87" s="6" t="s">
-        <v>577</v>
-      </c>
-      <c r="Q87" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="R87" s="5" t="s">
-        <v>534</v>
-      </c>
+        <v>558</v>
+      </c>
+      <c r="Q87" s="5"/>
+      <c r="R87" s="5"/>
     </row>
     <row r="88" spans="1:18" ht="18" customHeight="1">
       <c r="A88" s="5" t="s">
-        <v>578</v>
+        <v>22</v>
       </c>
       <c r="B88" s="5" t="s">
-        <v>579</v>
+        <v>559</v>
       </c>
       <c r="C88" s="5" t="s">
-        <v>580</v>
+        <v>560</v>
       </c>
       <c r="D88" s="5" t="s">
-        <v>581</v>
+        <v>561</v>
       </c>
       <c r="E88" s="5" t="s">
-        <v>539</v>
+        <v>562</v>
       </c>
       <c r="F88" s="5" t="s">
-        <v>582</v>
+        <v>563</v>
       </c>
       <c r="G88" s="6" t="s">
-        <v>583</v>
+        <v>120</v>
       </c>
       <c r="H88" s="9"/>
       <c r="I88" s="9"/>
@@ -6947,51 +7217,51 @@
         <v>28</v>
       </c>
       <c r="K88" s="5" t="s">
-        <v>39</v>
+        <v>88</v>
       </c>
       <c r="L88" s="5" t="s">
         <v>30</v>
       </c>
       <c r="M88" s="5" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="N88" s="5" t="s">
-        <v>473</v>
+        <v>109</v>
       </c>
       <c r="O88" s="5" t="s">
-        <v>584</v>
+        <v>564</v>
       </c>
       <c r="P88" s="6" t="s">
-        <v>585</v>
+        <v>565</v>
       </c>
       <c r="Q88" s="5" t="s">
         <v>102</v>
       </c>
       <c r="R88" s="5" t="s">
-        <v>534</v>
+        <v>103</v>
       </c>
     </row>
     <row r="89" spans="1:18" ht="18" customHeight="1">
       <c r="A89" s="5" t="s">
-        <v>22</v>
+        <v>67</v>
       </c>
       <c r="B89" s="5" t="s">
-        <v>579</v>
+        <v>559</v>
       </c>
       <c r="C89" s="5" t="s">
-        <v>586</v>
+        <v>560</v>
       </c>
       <c r="D89" s="5" t="s">
-        <v>587</v>
+        <v>566</v>
       </c>
       <c r="E89" s="5" t="s">
-        <v>529</v>
+        <v>562</v>
       </c>
       <c r="F89" s="5" t="s">
-        <v>588</v>
+        <v>563</v>
       </c>
       <c r="G89" s="6" t="s">
-        <v>589</v>
+        <v>499</v>
       </c>
       <c r="H89" s="9"/>
       <c r="I89" s="9"/>
@@ -6999,51 +7269,47 @@
         <v>28</v>
       </c>
       <c r="K89" s="5" t="s">
-        <v>39</v>
+        <v>88</v>
       </c>
       <c r="L89" s="5" t="s">
         <v>30</v>
       </c>
       <c r="M89" s="5" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="N89" s="5" t="s">
-        <v>473</v>
+        <v>109</v>
       </c>
       <c r="O89" s="5" t="s">
-        <v>590</v>
+        <v>564</v>
       </c>
       <c r="P89" s="6" t="s">
-        <v>591</v>
-      </c>
-      <c r="Q89" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="R89" s="5" t="s">
-        <v>534</v>
-      </c>
+        <v>567</v>
+      </c>
+      <c r="Q89" s="5"/>
+      <c r="R89" s="5"/>
     </row>
     <row r="90" spans="1:18" ht="18" customHeight="1">
       <c r="A90" s="5" t="s">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="B90" s="5" t="s">
-        <v>579</v>
+        <v>559</v>
       </c>
       <c r="C90" s="5" t="s">
-        <v>592</v>
+        <v>568</v>
       </c>
       <c r="D90" s="5" t="s">
-        <v>593</v>
+        <v>569</v>
       </c>
       <c r="E90" s="5" t="s">
-        <v>594</v>
+        <v>570</v>
       </c>
       <c r="F90" s="5" t="s">
-        <v>595</v>
+        <v>571</v>
       </c>
       <c r="G90" s="6" t="s">
-        <v>596</v>
+        <v>572</v>
       </c>
       <c r="H90" s="9"/>
       <c r="I90" s="9"/>
@@ -7051,151 +7317,155 @@
         <v>28</v>
       </c>
       <c r="K90" s="5" t="s">
-        <v>88</v>
+        <v>39</v>
       </c>
       <c r="L90" s="5" t="s">
         <v>30</v>
       </c>
       <c r="M90" s="5" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="N90" s="5" t="s">
-        <v>109</v>
+        <v>470</v>
       </c>
       <c r="O90" s="5" t="s">
-        <v>597</v>
+        <v>573</v>
       </c>
       <c r="P90" s="6" t="s">
-        <v>598</v>
+        <v>574</v>
       </c>
       <c r="Q90" s="5" t="s">
         <v>102</v>
       </c>
       <c r="R90" s="5" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
     </row>
     <row r="91" spans="1:18" ht="18" customHeight="1">
       <c r="A91" s="5" t="s">
-        <v>22</v>
+        <v>575</v>
       </c>
       <c r="B91" s="5" t="s">
+        <v>576</v>
+      </c>
+      <c r="C91" s="5" t="s">
+        <v>577</v>
+      </c>
+      <c r="D91" s="5" t="s">
+        <v>578</v>
+      </c>
+      <c r="E91" s="5" t="s">
+        <v>536</v>
+      </c>
+      <c r="F91" s="5" t="s">
         <v>579</v>
       </c>
-      <c r="C91" s="5" t="s">
-        <v>599</v>
-      </c>
-      <c r="D91" s="5" t="s">
-        <v>600</v>
-      </c>
-      <c r="E91" s="5" t="s">
-        <v>601</v>
-      </c>
-      <c r="F91" s="5" t="s">
-        <v>602</v>
-      </c>
       <c r="G91" s="6" t="s">
-        <v>603</v>
+        <v>580</v>
       </c>
       <c r="H91" s="9"/>
       <c r="I91" s="9"/>
       <c r="J91" s="5" t="s">
-        <v>98</v>
+        <v>28</v>
       </c>
       <c r="K91" s="5" t="s">
-        <v>88</v>
+        <v>39</v>
       </c>
       <c r="L91" s="5" t="s">
-        <v>132</v>
+        <v>30</v>
       </c>
       <c r="M91" s="5" t="s">
-        <v>339</v>
+        <v>528</v>
       </c>
       <c r="N91" s="5" t="s">
-        <v>109</v>
+        <v>470</v>
       </c>
       <c r="O91" s="5" t="s">
-        <v>604</v>
+        <v>581</v>
       </c>
       <c r="P91" s="6" t="s">
-        <v>605</v>
+        <v>582</v>
       </c>
       <c r="Q91" s="5" t="s">
         <v>102</v>
       </c>
       <c r="R91" s="5" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
     </row>
     <row r="92" spans="1:18" ht="18" customHeight="1">
       <c r="A92" s="5" t="s">
-        <v>67</v>
+        <v>22</v>
       </c>
       <c r="B92" s="5" t="s">
-        <v>579</v>
+        <v>576</v>
       </c>
       <c r="C92" s="5" t="s">
-        <v>599</v>
+        <v>583</v>
       </c>
       <c r="D92" s="5" t="s">
-        <v>606</v>
+        <v>584</v>
       </c>
       <c r="E92" s="5" t="s">
-        <v>601</v>
+        <v>526</v>
       </c>
       <c r="F92" s="5" t="s">
-        <v>602</v>
+        <v>585</v>
       </c>
       <c r="G92" s="6" t="s">
-        <v>607</v>
+        <v>586</v>
       </c>
       <c r="H92" s="9"/>
       <c r="I92" s="9"/>
       <c r="J92" s="5" t="s">
-        <v>98</v>
+        <v>28</v>
       </c>
       <c r="K92" s="5" t="s">
-        <v>88</v>
+        <v>39</v>
       </c>
       <c r="L92" s="5" t="s">
-        <v>132</v>
+        <v>30</v>
       </c>
       <c r="M92" s="5" t="s">
-        <v>339</v>
+        <v>528</v>
       </c>
       <c r="N92" s="5" t="s">
-        <v>109</v>
+        <v>470</v>
       </c>
       <c r="O92" s="5" t="s">
-        <v>604</v>
+        <v>587</v>
       </c>
       <c r="P92" s="6" t="s">
-        <v>608</v>
-      </c>
-      <c r="Q92" s="5"/>
-      <c r="R92" s="5"/>
+        <v>588</v>
+      </c>
+      <c r="Q92" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="R92" s="5" t="s">
+        <v>531</v>
+      </c>
     </row>
     <row r="93" spans="1:18" ht="18" customHeight="1">
       <c r="A93" s="5" t="s">
-        <v>67</v>
+        <v>22</v>
       </c>
       <c r="B93" s="5" t="s">
-        <v>609</v>
+        <v>576</v>
       </c>
       <c r="C93" s="5" t="s">
-        <v>610</v>
+        <v>589</v>
       </c>
       <c r="D93" s="5" t="s">
-        <v>611</v>
+        <v>590</v>
       </c>
       <c r="E93" s="5" t="s">
-        <v>612</v>
+        <v>591</v>
       </c>
       <c r="F93" s="5" t="s">
-        <v>613</v>
+        <v>592</v>
       </c>
       <c r="G93" s="6" t="s">
-        <v>614</v>
+        <v>593</v>
       </c>
       <c r="H93" s="9"/>
       <c r="I93" s="9"/>
@@ -7209,22 +7479,22 @@
         <v>30</v>
       </c>
       <c r="M93" s="5" t="s">
-        <v>615</v>
+        <v>528</v>
       </c>
       <c r="N93" s="5" t="s">
         <v>109</v>
       </c>
       <c r="O93" s="5" t="s">
-        <v>616</v>
+        <v>594</v>
       </c>
       <c r="P93" s="6" t="s">
-        <v>617</v>
+        <v>595</v>
       </c>
       <c r="Q93" s="5" t="s">
         <v>102</v>
       </c>
       <c r="R93" s="5" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
     </row>
     <row r="94" spans="1:18" ht="18" customHeight="1">
@@ -7232,111 +7502,263 @@
         <v>22</v>
       </c>
       <c r="B94" s="5" t="s">
-        <v>618</v>
+        <v>576</v>
       </c>
       <c r="C94" s="5" t="s">
-        <v>343</v>
+        <v>596</v>
       </c>
       <c r="D94" s="5" t="s">
-        <v>619</v>
+        <v>597</v>
       </c>
       <c r="E94" s="5" t="s">
-        <v>620</v>
+        <v>598</v>
       </c>
       <c r="F94" s="5" t="s">
-        <v>621</v>
+        <v>599</v>
       </c>
       <c r="G94" s="6" t="s">
-        <v>346</v>
-      </c>
-      <c r="H94" s="15">
-        <v>599.99</v>
-      </c>
-      <c r="I94" s="15" t="s">
-        <v>660</v>
-      </c>
+        <v>600</v>
+      </c>
+      <c r="H94" s="9"/>
+      <c r="I94" s="9"/>
       <c r="J94" s="5" t="s">
-        <v>48</v>
+        <v>98</v>
       </c>
       <c r="K94" s="5" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="L94" s="5" t="s">
-        <v>30</v>
+        <v>132</v>
       </c>
       <c r="M94" s="5" t="s">
+        <v>336</v>
+      </c>
+      <c r="N94" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="O94" s="5" t="s">
+        <v>601</v>
+      </c>
+      <c r="P94" s="6" t="s">
+        <v>602</v>
+      </c>
+      <c r="Q94" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="R94" s="5" t="s">
         <v>531</v>
       </c>
-      <c r="N94" s="5" t="s">
-        <v>274</v>
-      </c>
-      <c r="O94" s="5" t="s">
-        <v>622</v>
-      </c>
-      <c r="P94" s="6" t="s">
-        <v>623</v>
-      </c>
-      <c r="Q94" s="8" t="s">
-        <v>624</v>
-      </c>
-      <c r="R94" s="5" t="s">
-        <v>534</v>
-      </c>
-    </row>
-    <row r="95" spans="1:18">
+    </row>
+    <row r="95" spans="1:18" ht="18" customHeight="1">
       <c r="A95" s="5" t="s">
-        <v>22</v>
+        <v>67</v>
       </c>
       <c r="B95" s="5" t="s">
-        <v>618</v>
+        <v>576</v>
       </c>
       <c r="C95" s="5" t="s">
-        <v>625</v>
+        <v>596</v>
       </c>
       <c r="D95" s="5" t="s">
-        <v>626</v>
+        <v>603</v>
       </c>
       <c r="E95" s="5" t="s">
-        <v>620</v>
+        <v>598</v>
       </c>
       <c r="F95" s="5" t="s">
-        <v>627</v>
+        <v>599</v>
       </c>
       <c r="G95" s="6" t="s">
-        <v>628</v>
-      </c>
-      <c r="H95" s="15">
-        <v>249.99</v>
-      </c>
-      <c r="I95" s="15" t="s">
-        <v>655</v>
-      </c>
+        <v>604</v>
+      </c>
+      <c r="H95" s="9"/>
+      <c r="I95" s="9"/>
       <c r="J95" s="5" t="s">
-        <v>204</v>
+        <v>98</v>
       </c>
       <c r="K95" s="5" t="s">
-        <v>49</v>
+        <v>88</v>
       </c>
       <c r="L95" s="5" t="s">
         <v>132</v>
       </c>
       <c r="M95" s="5" t="s">
+        <v>336</v>
+      </c>
+      <c r="N95" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="O95" s="5" t="s">
+        <v>601</v>
+      </c>
+      <c r="P95" s="6" t="s">
+        <v>605</v>
+      </c>
+      <c r="Q95" s="5"/>
+      <c r="R95" s="5"/>
+    </row>
+    <row r="96" spans="1:18" ht="18" customHeight="1">
+      <c r="A96" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B96" s="5" t="s">
+        <v>606</v>
+      </c>
+      <c r="C96" s="5" t="s">
+        <v>607</v>
+      </c>
+      <c r="D96" s="5" t="s">
+        <v>608</v>
+      </c>
+      <c r="E96" s="5" t="s">
+        <v>609</v>
+      </c>
+      <c r="F96" s="5" t="s">
+        <v>610</v>
+      </c>
+      <c r="G96" s="6" t="s">
+        <v>611</v>
+      </c>
+      <c r="H96" s="9"/>
+      <c r="I96" s="9"/>
+      <c r="J96" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K96" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="L96" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="M96" s="5" t="s">
+        <v>612</v>
+      </c>
+      <c r="N96" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="O96" s="5" t="s">
+        <v>613</v>
+      </c>
+      <c r="P96" s="6" t="s">
+        <v>614</v>
+      </c>
+      <c r="Q96" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="R96" s="5" t="s">
         <v>531</v>
       </c>
-      <c r="N95" s="5" t="s">
+    </row>
+    <row r="97" spans="1:18" ht="18" customHeight="1">
+      <c r="A97" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B97" s="5" t="s">
+        <v>615</v>
+      </c>
+      <c r="C97" s="5" t="s">
+        <v>340</v>
+      </c>
+      <c r="D97" s="5" t="s">
+        <v>616</v>
+      </c>
+      <c r="E97" s="5" t="s">
+        <v>617</v>
+      </c>
+      <c r="F97" s="5" t="s">
+        <v>618</v>
+      </c>
+      <c r="G97" s="6" t="s">
+        <v>343</v>
+      </c>
+      <c r="H97" s="11">
+        <v>599.99</v>
+      </c>
+      <c r="I97" s="11" t="s">
+        <v>657</v>
+      </c>
+      <c r="J97" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="K97" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="L97" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="M97" s="5" t="s">
+        <v>528</v>
+      </c>
+      <c r="N97" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="O97" s="5" t="s">
+        <v>619</v>
+      </c>
+      <c r="P97" s="6" t="s">
+        <v>620</v>
+      </c>
+      <c r="Q97" s="8" t="s">
+        <v>621</v>
+      </c>
+      <c r="R97" s="5" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="98" spans="1:18">
+      <c r="A98" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B98" s="5" t="s">
+        <v>615</v>
+      </c>
+      <c r="C98" s="5" t="s">
+        <v>622</v>
+      </c>
+      <c r="D98" s="5" t="s">
+        <v>623</v>
+      </c>
+      <c r="E98" s="5" t="s">
+        <v>617</v>
+      </c>
+      <c r="F98" s="5" t="s">
+        <v>624</v>
+      </c>
+      <c r="G98" s="6" t="s">
+        <v>625</v>
+      </c>
+      <c r="H98" s="11">
+        <v>249.99</v>
+      </c>
+      <c r="I98" s="11" t="s">
+        <v>652</v>
+      </c>
+      <c r="J98" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="K98" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="L98" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="M98" s="5" t="s">
+        <v>528</v>
+      </c>
+      <c r="N98" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="O95" s="5" t="s">
-        <v>629</v>
-      </c>
-      <c r="P95" s="6" t="s">
-        <v>630</v>
-      </c>
-      <c r="Q95" s="8" t="s">
-        <v>631</v>
-      </c>
-      <c r="R95" s="5" t="s">
-        <v>534</v>
+      <c r="O98" s="5" t="s">
+        <v>626</v>
+      </c>
+      <c r="P98" s="6" t="s">
+        <v>627</v>
+      </c>
+      <c r="Q98" s="8" t="s">
+        <v>628</v>
+      </c>
+      <c r="R98" s="5" t="s">
+        <v>531</v>
       </c>
     </row>
   </sheetData>
@@ -7357,6 +7779,7 @@
     <hyperlink ref="P7" r:id="rId8" xr:uid="{92AB9D3B-E263-1644-BF94-1DA28A008093}"/>
     <hyperlink ref="Q7" r:id="rId9" xr:uid="{65199225-5275-A045-A41A-38A05ADABDAA}"/>
     <hyperlink ref="P35" r:id="rId10" xr:uid="{9F1B81DE-A706-0140-B404-AD34667BAD93}"/>
+    <hyperlink ref="Q50" r:id="rId11" xr:uid="{E28E6611-8825-4B44-BAEB-BCD7296741B2}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>